<commit_message>
Update test results - 2026-06-22 18:06:44
</commit_message>
<xml_diff>
--- a/best-configs_results.xlsx
+++ b/best-configs_results.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ⛓️</t>
+          <t xml:space="preserve"> By EbraSha 🕷️</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -507,17 +507,17 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>r3mrcg001269pz2.cybervena.com:50099</t>
+          <t>ru.moktana.app:51523</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>218.8</t>
+          <t>225.4</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>309.6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -527,17 +527,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>207.3</t>
+          <t>217.2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>230.3</t>
+          <t>233.6</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>42.55</t>
+          <t>42.19</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧠</t>
+          <t xml:space="preserve"> By EbraSha 🤖</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -563,17 +563,17 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45.129.96.62:41348</t>
+          <t>61.171.92.202:1001</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>253.9</t>
+          <t>265.9</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1159.1</t>
+          <t>298.9</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -583,17 +583,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>248.4</t>
+          <t>218.2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>259.4</t>
+          <t>313.5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>38.22</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 👑</t>
+          <t xml:space="preserve"> By EbraSha 🚨</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -619,17 +619,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>66.70.190.236:41344</t>
+          <t>103.130.147.40:1122</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>269.8</t>
+          <t>339.9</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>63.4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,17 +639,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>266.8</t>
+          <t>200.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>272.7</t>
+          <t>479.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>36.51</t>
+          <t>18.60</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🦈</t>
+          <t xml:space="preserve"> By EbraSha 📀</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -675,12 +675,12 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>91.208.75.251:3478</t>
+          <t>email protected:8388</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>294.5</t>
+          <t>404.5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>270.9</t>
+          <t>271.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>318.0</t>
+          <t>537.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>30.51</t>
+          <t>16.89</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 📀</t>
+          <t xml:space="preserve"> By EbraSha 🖥️</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -731,12 +731,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>94.131.127.154:48877</t>
+          <t>email protected:30129</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>308.2</t>
+          <t>414.3</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -751,17 +751,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>269.5</t>
+          <t>286.3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>346.9</t>
+          <t>542.3</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>27.55</t>
+          <t>16.80</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -776,28 +776,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕶️</t>
+          <t>@FarazV2ray</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>46.246.97.3:31348</t>
+          <t>209.127.228.114:443</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>317.8</t>
+          <t>431.4</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>141.4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -807,17 +807,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>289.2</t>
+          <t>407.1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>346.5</t>
+          <t>455.8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>27.91</t>
+          <t>21.47</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -832,28 +832,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ⚙️</t>
+          <t>🎭</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>108.181.121.226:8388</t>
+          <t>159.195.44.159:443</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>322.7</t>
+          <t>448.4</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>150.8</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -863,17 +863,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>289.9</t>
+          <t>425.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>355.6</t>
+          <t>471.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>27.09</t>
+          <t>20.81</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🥷</t>
+          <t xml:space="preserve"> By EbraSha 🕹️</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -899,17 +899,17 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>47.80.24.245:8127</t>
+          <t>82.38.31.16:8080</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>384.2</t>
+          <t>465.7</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>163.8</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -919,17 +919,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>251.7</t>
+          <t>200.7</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>516.7</t>
+          <t>730.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>17.49</t>
+          <t>11.90</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -944,28 +944,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕷️</t>
+          <t>🚀</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2a00:b700:2::23c:443</t>
+          <t>89.124.119.209:443</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>453.7</t>
+          <t>592.4</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>148.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -975,17 +975,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>212.7</t>
+          <t>567.4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>694.7</t>
+          <t>617.3</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>12.59</t>
+          <t>15.93</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1000,28 +1000,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧲</t>
+          <t>57.🇬🇧Великобритания | @LimeVPNFREE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2a0b:8bc0:2:856::1:443</t>
+          <t>209.127.228.114:443</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>550.3</t>
+          <t>675.5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>139.3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1031,17 +1031,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>465.7</t>
+          <t>487.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>635.0</t>
+          <t>863.2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>14.92</t>
+          <t>10.63</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧲</t>
+          <t xml:space="preserve"> By EbraSha 🌐</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1067,17 +1067,17 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>r3mrcg001269pz2.cybervena.com:50099</t>
+          <t>82.38.31.17:8080</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>799.0</t>
+          <t>684.1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>161.8</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1087,17 +1087,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>276.3</t>
+          <t>207.5</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1321.8</t>
+          <t>1160.6</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>7.36</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1112,28 +1112,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌑</t>
+          <t>53.🇳🇱Нидерланды | @LimeVPNFREE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ru.moktana.app:51523</t>
+          <t>89.124.90.42:443</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>806.4</t>
+          <t>706.8</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>726.0</t>
+          <t>132.8</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1143,17 +1143,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>290.8</t>
+          <t>431.8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1322.1</t>
+          <t>981.9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>6.51</t>
+          <t>9.13</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 📀</t>
+          <t xml:space="preserve"> By EbraSha 📛</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1179,17 +1179,17 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>email protected:17276</t>
+          <t>ru.moktana.app:51523</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1120.0</t>
+          <t>749.1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>298.0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1199,17 +1199,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>271.6</t>
+          <t>545.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1968.4</t>
+          <t>952.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>4.31</t>
+          <t>9.65</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1224,12 +1224,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🔐</t>
+          <t xml:space="preserve"> By EbraSha 🌀</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1155.9</t>
+          <t>785.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1255,17 +1255,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>246.3</t>
+          <t>325.1</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2065.5</t>
+          <t>1244.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>6.97</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧲</t>
+          <t xml:space="preserve"> By EbraSha 🧠</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1291,17 +1291,17 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>141.227.152.129:8388</t>
+          <t>r3mrcg001286ek2.cybervena.com:50099</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1207.2</t>
+          <t>923.1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>167.6</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1311,17 +1311,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>277.0</t>
+          <t>213.9</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2137.4</t>
+          <t>1632.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>3.96</t>
+          <t>5.19</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1336,28 +1336,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>🇸🇪SE-🚀@V2Ray_Hub1200</t>
+          <t xml:space="preserve"> By EbraSha 🐺</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>se.faygo.bot:443</t>
+          <t>2605:e440:15::12d:443</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1236.9</t>
+          <t>956.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>146.6</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1367,17 +1367,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1060.2</t>
+          <t>282.7</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>1413.5</t>
+          <t>1629.3</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>6.73</t>
+          <t>5.24</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1392,23 +1392,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌑</t>
+          <t xml:space="preserve"> By EbraSha 🦅</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2401:c080:3800:3efd:5400:6ff:fe40:972b:443</t>
+          <t>148.253.208.76:3478</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1725.1</t>
+          <t>959.4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1423,17 +1423,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1433.7</t>
+          <t>550.1</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2016.6</t>
+          <t>1368.8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>4.68</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1448,23 +1448,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🔌</t>
+          <t xml:space="preserve"> By EbraSha 🚧</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2605:e440:10::1:68:443</t>
+          <t>161.129.71.148:17913</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1735.8</t>
+          <t>975.2</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1479,17 +1479,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1464.2</t>
+          <t>261.1</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2007.4</t>
+          <t>1689.3</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.72</t>
+          <t>5.04</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1504,28 +1504,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ✨</t>
+          <t xml:space="preserve"> By EbraSha 🚧</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>103.130.147.40:1122</t>
+          <t>email protected:443</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1747.8</t>
+          <t>991.4</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>771.6</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>280.1</t>
+          <t>227.9</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3215.5</t>
+          <t>1754.8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2.62</t>
+          <t>4.83</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>By EbraSha 🪐</t>
+          <t>By EbraSha 🃏</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1575,17 +1575,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>163.223.224.68:49515</t>
+          <t>186.244.208.78:30022</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1865.7</t>
+          <t>1095.2</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>333.9</t>
+          <t>290.5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1595,17 +1595,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1839.7</t>
+          <t>596.9</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1891.7</t>
+          <t>1593.5</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>5.26</t>
+          <t>5.56</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">

</xml_diff>

<commit_message>
Update test results - 2026-06-22 18:26:48
</commit_message>
<xml_diff>
--- a/best-configs_results.xlsx
+++ b/best-configs_results.xlsx
@@ -496,28 +496,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕷️</t>
+          <t>By EbraSha 🦅</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>vmess</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DE (Germany)</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ru.moktana.app:51523</t>
+          <t>89.167.82.102:4443</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>225.4</t>
+          <t>534.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>309.6</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -527,17 +531,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>217.2</t>
+          <t>448.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>233.6</t>
+          <t>619.1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>42.19</t>
+          <t>15.28</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -552,28 +556,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🤖</t>
+          <t xml:space="preserve"> By EbraSha ⌨️</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>61.171.92.202:1001</t>
+          <t>62.60.155.0:443</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>265.9</t>
+          <t>959.4</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>298.9</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -583,17 +587,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>218.2</t>
+          <t>613.5</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>313.5</t>
+          <t>1305.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>6.90</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -608,28 +612,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🚨</t>
+          <t>By EbraSha 🕷️</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>vmess</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DE (Germany)</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>103.130.147.40:1122</t>
+          <t>89.167.82.102:4443</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>339.9</t>
+          <t>971.7</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>63.4</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,17 +647,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>200.1</t>
+          <t>479.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>479.7</t>
+          <t>1464.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>18.60</t>
+          <t>5.99</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -664,28 +672,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 📀</t>
+          <t xml:space="preserve"> By EbraSha 🌐</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>vless</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PL (Poland)</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>email protected:8388</t>
+          <t>144.31.241.7:8443</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>404.5</t>
+          <t>1152.2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -695,17 +707,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>271.8</t>
+          <t>591.7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>537.2</t>
+          <t>1712.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>16.89</t>
+          <t>5.14</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -720,28 +732,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🖥️</t>
+          <t xml:space="preserve"> By EbraSha 🌍</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>vless</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DE (Germany)</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>email protected:30129</t>
+          <t>159.195.148.47:443</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>414.3</t>
+          <t>1190.1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -751,17 +767,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>286.3</t>
+          <t>631.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>542.3</t>
+          <t>1748.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>16.80</t>
+          <t>5.05</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -776,28 +792,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>@FarazV2ray</t>
+          <t>By EbraSha 🪬</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>vless</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>vmess</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>US (United States)</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>209.127.228.114:443</t>
+          <t>186.244.208.78:30022</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>431.4</t>
+          <t>1207.1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>141.4</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -807,17 +827,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>407.1</t>
+          <t>719.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>455.8</t>
+          <t>1694.9</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>21.47</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -832,7 +852,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>🎭</t>
+          <t>🚀</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -843,17 +863,17 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>159.195.44.159:443</t>
+          <t>89.124.119.209:443</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>448.4</t>
+          <t>1295.1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>150.8</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -863,17 +883,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>425.7</t>
+          <t>746.6</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>471.0</t>
+          <t>1843.5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>20.81</t>
+          <t>4.83</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -888,28 +908,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕹️</t>
+          <t>By EbraSha 🧠</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>vmess</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DE (Germany)</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>82.38.31.16:8080</t>
+          <t>89.167.82.102:8880</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>465.7</t>
+          <t>1405.4</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>163.8</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -919,17 +943,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>200.7</t>
+          <t>448.4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>730.7</t>
+          <t>2362.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>11.90</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -944,28 +968,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>🚀</t>
+          <t xml:space="preserve"> By EbraSha 🛜</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>89.124.119.209:443</t>
+          <t>46.246.97.3:31348</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>592.4</t>
+          <t>1412.6</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>148.5</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -975,17 +999,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>567.4</t>
+          <t>788.8</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>617.3</t>
+          <t>2036.4</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>15.93</t>
+          <t>4.36</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1000,7 +1024,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>57.🇬🇧Великобритания | @LimeVPNFREE</t>
+          <t>70.🌐Неизвестно | @LimeVPNFREE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1011,17 +1035,17 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>209.127.228.114:443</t>
+          <t>193.233.82.126:443</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>675.5</t>
+          <t>1423.7</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>139.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1031,17 +1055,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>487.8</t>
+          <t>1114.9</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>863.2</t>
+          <t>1732.5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>10.63</t>
+          <t>5.38</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1056,28 +1080,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌐</t>
+          <t xml:space="preserve"> By EbraSha 🚧</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>82.38.31.17:8080</t>
+          <t>77.73.131.154:443</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>684.1</t>
+          <t>1486.3</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>161.8</t>
+          <t>25.7</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1087,17 +1111,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>207.5</t>
+          <t>741.8</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1160.6</t>
+          <t>2230.9</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>7.36</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1112,7 +1136,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>53.🇳🇱Нидерланды | @LimeVPNFREE</t>
+          <t xml:space="preserve"> By EbraSha 🧨</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1120,20 +1144,24 @@
           <t>vless</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>US (United States)</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>89.124.90.42:443</t>
+          <t>82.21.92.47:9443</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>706.8</t>
+          <t>1487.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>132.8</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1143,17 +1171,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>431.8</t>
+          <t>926.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>981.9</t>
+          <t>2047.6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>9.13</t>
+          <t>4.39</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1168,28 +1196,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 📛</t>
+          <t xml:space="preserve"> By EbraSha 🛸</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>vless</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ru.moktana.app:51523</t>
+          <t>45.89.106.101:40443</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>749.1</t>
+          <t>1487.3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>298.0</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1199,17 +1231,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>545.8</t>
+          <t>1337.2</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>952.5</t>
+          <t>1637.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>9.65</t>
+          <t>5.88</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1224,12 +1256,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌀</t>
+          <t xml:space="preserve"> By EbraSha ✨</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1240,7 +1272,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>785.0</t>
+          <t>1490.3</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1255,17 +1287,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>325.1</t>
+          <t>837.6</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1244.8</t>
+          <t>2143.1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>6.97</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1280,28 +1312,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧠</t>
+          <t xml:space="preserve"> By EbraSha 🌀</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>r3mrcg001286ek2.cybervena.com:50099</t>
+          <t>vpnv1.aspidnet.xyz:443</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>923.1</t>
+          <t>1511.7</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>81.0</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1311,17 +1343,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>213.9</t>
+          <t>1487.9</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>1632.4</t>
+          <t>1535.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>5.19</t>
+          <t>6.47</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1336,28 +1368,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🐺</t>
+          <t xml:space="preserve"> By EbraSha ⌨️</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2605:e440:15::12d:443</t>
+          <t>r3mrcg001269pz2.cybervena.com:50099</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>956.0</t>
+          <t>1511.8</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1367,17 +1399,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>282.7</t>
+          <t>639.4</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>1629.3</t>
+          <t>2384.2</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>3.64</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1392,7 +1424,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🦅</t>
+          <t xml:space="preserve"> By EbraSha 🚀</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1403,17 +1435,17 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>148.253.208.76:3478</t>
+          <t>series-a1.samanehha.co:443</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>959.4</t>
+          <t>1538.9</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1423,17 +1455,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>550.1</t>
+          <t>699.3</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>1368.8</t>
+          <t>2378.6</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1448,7 +1480,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🚧</t>
+          <t xml:space="preserve"> By EbraSha 🌌</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1459,17 +1491,17 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>161.129.71.148:17913</t>
+          <t>admin.c1.webramz.co:443</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>975.2</t>
+          <t>1566.1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1479,17 +1511,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>261.1</t>
+          <t>668.9</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1689.3</t>
+          <t>2463.2</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>5.04</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1504,23 +1536,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🚧</t>
+          <t xml:space="preserve"> By EbraSha 🕷️</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>email protected:443</t>
+          <t>2401:c080:1c00:21dd:5400:6ff:fe43:2737:443</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>991.4</t>
+          <t>1596.4</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1535,17 +1567,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>227.9</t>
+          <t>758.4</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1754.8</t>
+          <t>2434.4</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>4.83</t>
+          <t>3.60</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1560,32 +1592,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>By EbraSha 🃏</t>
+          <t>79.🌐Неизвестно | @LimeVPNFREE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>vmess</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>vless</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>186.244.208.78:30022</t>
+          <t>77.246.109.191:34045</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1095.2</t>
+          <t>1633.8</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>290.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1595,17 +1623,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>596.9</t>
+          <t>1560.4</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1593.5</t>
+          <t>1707.3</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>5.56</t>
+          <t>5.75</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">

</xml_diff>

<commit_message>
Update test results - 2026-06-22 18:28:06
</commit_message>
<xml_diff>
--- a/best-configs_results.xlsx
+++ b/best-configs_results.xlsx
@@ -496,32 +496,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>By EbraSha 🦅</t>
+          <t xml:space="preserve"> By EbraSha 🔐</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>vmess</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DE (Germany)</t>
-        </is>
-      </c>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>89.167.82.102:4443</t>
+          <t>45.129.96.62:41348</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>534.0</t>
+          <t>306.7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>669.5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -531,17 +527,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>448.8</t>
+          <t>280.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>619.1</t>
+          <t>332.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>15.28</t>
+          <t>29.12</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -556,28 +552,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ⌨️</t>
+          <t xml:space="preserve"> By EbraSha ♠️</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>62.60.155.0:443</t>
+          <t>161.129.71.148:17913</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>959.4</t>
+          <t>324.7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -587,17 +583,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>613.5</t>
+          <t>297.9</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1305.4</t>
+          <t>351.5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>6.90</t>
+          <t>27.58</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -612,32 +608,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>By EbraSha 🕷️</t>
+          <t xml:space="preserve"> By EbraSha ⌨️</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>vmess</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DE (Germany)</t>
-        </is>
-      </c>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>89.167.82.102:4443</t>
+          <t>207.2.120.46:3478</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>971.7</t>
+          <t>385.3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -647,17 +639,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>479.1</t>
+          <t>223.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1464.2</t>
+          <t>547.6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>5.99</t>
+          <t>16.27</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -672,7 +664,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌐</t>
+          <t>🎭</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -680,24 +672,20 @@
           <t>vless</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>PL (Poland)</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>144.31.241.7:8443</t>
+          <t>159.195.44.159:443</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1152.2</t>
+          <t>408.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>112.7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -707,17 +695,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>591.7</t>
+          <t>403.5</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1712.7</t>
+          <t>412.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>5.14</t>
+          <t>24.13</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -732,32 +720,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌍</t>
+          <t xml:space="preserve"> By EbraSha 🗿</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>vless</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>DE (Germany)</t>
-        </is>
-      </c>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>159.195.148.47:443</t>
+          <t>103.130.147.40:1122</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1190.1</t>
+          <t>417.9</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>97.6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -767,17 +751,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>631.4</t>
+          <t>312.3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1748.8</t>
+          <t>523.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>5.05</t>
+          <t>17.63</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -792,32 +776,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>By EbraSha 🪬</t>
+          <t xml:space="preserve"> By EbraSha ⌨️</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>vmess</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>US (United States)</t>
-        </is>
-      </c>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>186.244.208.78:30022</t>
+          <t>r3mrcg001269pz2.cybervena.com:50099</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1207.1</t>
+          <t>431.8</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -827,17 +807,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>719.3</t>
+          <t>305.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1694.9</t>
+          <t>557.8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>5.27</t>
+          <t>16.39</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -852,28 +832,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>🚀</t>
+          <t xml:space="preserve"> By EbraSha 🕷️</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>89.124.119.209:443</t>
+          <t>61.171.92.202:1001</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1295.1</t>
+          <t>498.9</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>347.1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -883,17 +863,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>746.6</t>
+          <t>363.4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1843.5</t>
+          <t>634.3</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>4.83</t>
+          <t>14.48</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -908,32 +888,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>By EbraSha 🧠</t>
+          <t>@FarazV2ray</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>vmess</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>DE (Germany)</t>
-        </is>
-      </c>
+          <t>vless</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>89.167.82.102:8880</t>
+          <t>209.127.228.114:443</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1405.4</t>
+          <t>530.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>138.0</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -943,17 +919,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>448.4</t>
+          <t>432.5</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2362.5</t>
+          <t>627.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>14.97</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -968,7 +944,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🛜</t>
+          <t xml:space="preserve"> By EbraSha 🧪</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -979,17 +955,17 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>46.246.97.3:31348</t>
+          <t>email protected:17276</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1412.6</t>
+          <t>543.3</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -999,17 +975,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>788.8</t>
+          <t>182.4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2036.4</t>
+          <t>904.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>4.36</t>
+          <t>9.49</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1024,28 +1000,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>70.🌐Неизвестно | @LimeVPNFREE</t>
+          <t xml:space="preserve"> By EbraSha 🪬</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>193.233.82.126:443</t>
+          <t>91.208.75.251:3478</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1423.7</t>
+          <t>611.5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1055,17 +1031,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1114.9</t>
+          <t>546.5</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1732.5</t>
+          <t>676.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>5.38</t>
+          <t>14.22</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1080,28 +1056,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🚧</t>
+          <t xml:space="preserve"> By EbraSha 🕶️</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>77.73.131.154:443</t>
+          <t>47.80.24.245:8127</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1486.3</t>
+          <t>612.6</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>25.7</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1111,17 +1087,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>741.8</t>
+          <t>529.5</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2230.9</t>
+          <t>695.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>3.94</t>
+          <t>13.70</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1136,7 +1112,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧨</t>
+          <t>🚀</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1144,24 +1120,20 @@
           <t>vless</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>US (United States)</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>82.21.92.47:9443</t>
+          <t>89.124.119.209:443</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1487.0</t>
+          <t>628.9</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>123.6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1171,17 +1143,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>926.3</t>
+          <t>548.8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2047.6</t>
+          <t>708.9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>4.39</t>
+          <t>13.48</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1201,27 +1173,23 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>vless</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>45.89.106.101:40443</t>
+          <t>45.129.96.62:41348</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1487.3</t>
+          <t>686.5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>671.1</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1231,17 +1199,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1337.2</t>
+          <t>522.6</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1637.4</t>
+          <t>850.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>5.88</t>
+          <t>10.89</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1256,28 +1224,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ✨</t>
+          <t>𝗝𝗼𝗶𝗻 ➠ @MoOon_proxy 6`</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>email protected:443</t>
+          <t>tg.riotvpn.eu:443</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1490.3</t>
+          <t>807.2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1775.7</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1287,17 +1255,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>837.6</t>
+          <t>784.8</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2143.1</t>
+          <t>829.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>11.92</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1312,7 +1280,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌀</t>
+          <t xml:space="preserve"> By EbraSha ♣️</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1320,20 +1288,24 @@
           <t>vless</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>vpnv1.aspidnet.xyz:443</t>
+          <t>178.236.17.86:443</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1511.7</t>
+          <t>849.3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>332.9</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1343,17 +1315,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1487.9</t>
+          <t>786.4</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>1535.4</t>
+          <t>912.3</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>6.47</t>
+          <t>10.66</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1368,28 +1340,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ⌨️</t>
+          <t>@BESTIIVPNBOT خرید سرور اختصاصی 💲</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>r3mrcg001269pz2.cybervena.com:50099</t>
+          <t>fi.faygo.bot:443</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1511.8</t>
+          <t>869.4</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>126.9</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1399,17 +1371,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>639.4</t>
+          <t>644.5</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2384.2</t>
+          <t>1094.2</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>3.64</t>
+          <t>8.42</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1424,28 +1396,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🚀</t>
+          <t xml:space="preserve"> By EbraSha 🔋</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>series-a1.samanehha.co:443</t>
+          <t>2a0b:8bc0:2:856::1:443</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1538.9</t>
+          <t>879.5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1455,17 +1427,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>699.3</t>
+          <t>260.7</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2378.6</t>
+          <t>1498.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>3.67</t>
+          <t>5.70</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1480,7 +1452,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌌</t>
+          <t xml:space="preserve"> By EbraSha 💻</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1491,17 +1463,17 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>admin.c1.webramz.co:443</t>
+          <t>r3mrcg001286ek2.cybervena.com:50099</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1566.1</t>
+          <t>906.9</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>223.1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1511,17 +1483,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>668.9</t>
+          <t>446.7</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2463.2</t>
+          <t>1367.1</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>6.42</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1536,23 +1508,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕷️</t>
+          <t xml:space="preserve"> By EbraSha 🌪️</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2401:c080:1c00:21dd:5400:6ff:fe43:2737:443</t>
+          <t>email protected:443</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1596.4</t>
+          <t>916.2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1567,17 +1539,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>758.4</t>
+          <t>551.1</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2434.4</t>
+          <t>1281.3</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>6.98</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1592,28 +1564,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>79.🌐Неизвестно | @LimeVPNFREE</t>
+          <t xml:space="preserve"> By EbraSha 🧪</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>77.246.109.191:34045</t>
+          <t>email protected:1001</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1633.8</t>
+          <t>989.4</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1623,17 +1595,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1560.4</t>
+          <t>202.2</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1707.3</t>
+          <t>1776.6</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>5.75</t>
+          <t>4.76</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">

</xml_diff>

<commit_message>
Update test results - 2026-06-22 18:35:43
</commit_message>
<xml_diff>
--- a/best-configs_results.xlsx
+++ b/best-configs_results.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🔐</t>
+          <t xml:space="preserve"> By EbraSha 🃏</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -507,17 +507,17 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>45.129.96.62:41348</t>
+          <t>141.227.152.129:8388</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>306.7</t>
+          <t>569.4</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>669.5</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -527,17 +527,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>280.8</t>
+          <t>560.9</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>332.7</t>
+          <t>578.0</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>29.12</t>
+          <t>17.20</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ♠️</t>
+          <t xml:space="preserve"> By EbraSha 🛸</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -563,17 +563,17 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>161.129.71.148:17913</t>
+          <t>185.202.93.194:41348</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>324.7</t>
+          <t>611.4</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -583,17 +583,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>297.9</t>
+          <t>587.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>351.5</t>
+          <t>635.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>27.58</t>
+          <t>15.49</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ⌨️</t>
+          <t xml:space="preserve"> By EbraSha 🐺</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -619,17 +619,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>207.2.120.46:3478</t>
+          <t>94.131.127.154:48877</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>385.3</t>
+          <t>633.9</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>13.6</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,17 +639,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>223.1</t>
+          <t>604.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>547.6</t>
+          <t>663.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>16.27</t>
+          <t>14.80</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -664,28 +664,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>🎭</t>
+          <t xml:space="preserve"> By EbraSha 📶</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>159.195.44.159:443</t>
+          <t>email protected:443</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>408.0</t>
+          <t>636.2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>112.7</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>403.5</t>
+          <t>634.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>412.5</t>
+          <t>638.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>24.13</t>
+          <t>15.65</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🗿</t>
+          <t xml:space="preserve"> By EbraSha 🧠</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -731,17 +731,17 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>103.130.147.40:1122</t>
+          <t>91.208.75.251:3478</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>417.9</t>
+          <t>647.6</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>97.6</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -751,17 +751,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>312.3</t>
+          <t>577.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>523.5</t>
+          <t>717.6</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>17.63</t>
+          <t>13.39</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ⌨️</t>
+          <t xml:space="preserve"> By EbraSha 🖥️</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -787,17 +787,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>r3mrcg001269pz2.cybervena.com:50099</t>
+          <t>140.174.184.5:8388</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>431.8</t>
+          <t>662.9</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>14.8</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -807,17 +807,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>305.8</t>
+          <t>636.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>557.8</t>
+          <t>689.5</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>16.39</t>
+          <t>14.28</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -832,28 +832,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕷️</t>
+          <t>By EbraSha 🕶️</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ss</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>vmess</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DE (Germany)</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>61.171.92.202:1001</t>
+          <t>89.167.82.102:4443</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>498.9</t>
+          <t>668.2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>347.1</t>
+          <t>28.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -863,17 +867,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>363.4</t>
+          <t>389.8</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>634.3</t>
+          <t>946.6</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>14.48</t>
+          <t>9.42</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -888,28 +892,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>@FarazV2ray</t>
+          <t>By EbraSha 🚧</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>vless</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>vmess</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DE (Germany)</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>209.127.228.114:443</t>
+          <t>89.167.82.102:4443</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>530.0</t>
+          <t>670.2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>138.0</t>
+          <t>30.7</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -919,17 +927,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>432.5</t>
+          <t>412.5</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>627.5</t>
+          <t>927.9</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>14.97</t>
+          <t>9.67</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -944,7 +952,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧪</t>
+          <t xml:space="preserve"> By EbraSha 🔮</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -955,17 +963,17 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>email protected:17276</t>
+          <t>68.168.209.194:17276</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>543.3</t>
+          <t>673.2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>5.9</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -975,17 +983,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>182.4</t>
+          <t>617.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>904.1</t>
+          <t>728.6</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9.49</t>
+          <t>13.30</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1000,7 +1008,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🪬</t>
+          <t xml:space="preserve"> By EbraSha 📱</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1011,17 +1019,17 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>91.208.75.251:3478</t>
+          <t>82.38.31.2:8080</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>611.5</t>
+          <t>681.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1031,17 +1039,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>546.5</t>
+          <t>575.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>676.4</t>
+          <t>786.3</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>14.22</t>
+          <t>12.05</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1056,28 +1064,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕶️</t>
+          <t xml:space="preserve"> By EbraSha 🦈</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>47.80.24.245:8127</t>
+          <t>109.73.65.116:493</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>612.6</t>
+          <t>728.6</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1087,17 +1095,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>529.5</t>
+          <t>628.8</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>695.7</t>
+          <t>828.5</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>13.70</t>
+          <t>11.50</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1112,28 +1120,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>🚀</t>
+          <t xml:space="preserve"> By EbraSha 🩸</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>89.124.119.209:443</t>
+          <t>161.129.71.148:17913</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>628.9</t>
+          <t>751.3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>123.6</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1143,17 +1151,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>548.8</t>
+          <t>707.5</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>708.9</t>
+          <t>795.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>13.48</t>
+          <t>12.30</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1168,7 +1176,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🛸</t>
+          <t xml:space="preserve"> By EbraSha 🥷</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1179,17 +1187,17 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>45.129.96.62:41348</t>
+          <t>168.138.175.92:9888</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>686.5</t>
+          <t>760.8</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>671.1</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1199,17 +1207,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>522.6</t>
+          <t>712.7</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>850.4</t>
+          <t>809.0</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>10.89</t>
+          <t>12.06</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1224,28 +1232,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>𝗝𝗼𝗶𝗻 ➠ @MoOon_proxy 6`</t>
+          <t xml:space="preserve"> By EbraSha 🔐</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>tg.riotvpn.eu:443</t>
+          <t>email protected:1001</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>807.2</t>
+          <t>808.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1775.7</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1255,17 +1263,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>784.8</t>
+          <t>555.7</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>829.7</t>
+          <t>1060.2</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>11.92</t>
+          <t>8.59</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1280,32 +1288,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha ♣️</t>
+          <t xml:space="preserve"> By EbraSha 🕶️</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>vless</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>178.236.17.86:443</t>
+          <t>email protected:8388</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>849.3</t>
+          <t>808.1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>332.9</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1315,17 +1319,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>786.4</t>
+          <t>705.1</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>912.3</t>
+          <t>911.2</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>10.66</t>
+          <t>10.48</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1340,7 +1344,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>@BESTIIVPNBOT خرید سرور اختصاصی 💲</t>
+          <t xml:space="preserve"> By EbraSha 🚀</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1351,17 +1355,17 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>fi.faygo.bot:443</t>
+          <t>185.68.185.212:50029</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>869.4</t>
+          <t>810.3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>126.9</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1371,17 +1375,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>644.5</t>
+          <t>784.8</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>1094.2</t>
+          <t>835.8</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>8.42</t>
+          <t>11.82</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1396,23 +1400,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🔋</t>
+          <t xml:space="preserve"> By EbraSha 🐺</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2a0b:8bc0:2:856::1:443</t>
+          <t>email protected:30129</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>879.5</t>
+          <t>823.2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1427,17 +1431,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>260.7</t>
+          <t>743.9</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>1498.4</t>
+          <t>902.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.70</t>
+          <t>10.69</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1452,7 +1456,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 💻</t>
+          <t xml:space="preserve"> By EbraSha 🧩</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1463,17 +1467,17 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>r3mrcg001286ek2.cybervena.com:50099</t>
+          <t>78.129.155.63:3030</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>906.9</t>
+          <t>857.2</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>223.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1483,17 +1487,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>446.7</t>
+          <t>576.4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1367.1</t>
+          <t>1138.0</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>6.42</t>
+          <t>7.97</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1508,28 +1512,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🌪️</t>
+          <t xml:space="preserve"> By EbraSha 🦅</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>email protected:443</t>
+          <t>77.73.131.154:443</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>916.2</t>
+          <t>907.8</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1539,17 +1543,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>551.1</t>
+          <t>680.4</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1281.3</t>
+          <t>1135.3</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>6.98</t>
+          <t>8.13</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1564,28 +1568,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧪</t>
+          <t>🎭</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>email protected:1001</t>
+          <t>159.195.44.159:443</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>989.4</t>
+          <t>920.1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1595,17 +1599,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>202.2</t>
+          <t>670.4</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1776.6</t>
+          <t>1169.8</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>4.76</t>
+          <t>7.85</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">

</xml_diff>

<commit_message>
Update test results - 2026-06-22 18:37:19
</commit_message>
<xml_diff>
--- a/best-configs_results.xlsx
+++ b/best-configs_results.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🃏</t>
+          <t xml:space="preserve"> By EbraSha ♠️</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -507,17 +507,17 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>141.227.152.129:8388</t>
+          <t>r3mrcg001269pz2.cybervena.com:50099</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>569.4</t>
+          <t>237.8</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -527,17 +527,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>560.9</t>
+          <t>213.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>578.0</t>
+          <t>262.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>17.20</t>
+          <t>36.71</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🛸</t>
+          <t xml:space="preserve"> By EbraSha 🧿</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -563,17 +563,17 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>185.202.93.194:41348</t>
+          <t>ru.moktana.app:51523</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>611.4</t>
+          <t>248.2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>101.6</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -583,17 +583,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>587.4</t>
+          <t>234.1</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>635.4</t>
+          <t>262.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>15.49</t>
+          <t>37.30</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🐺</t>
+          <t xml:space="preserve"> By EbraSha 🛸</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -619,17 +619,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>94.131.127.154:48877</t>
+          <t>185.202.93.194:41348</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>633.9</t>
+          <t>319.5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>13.6</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,17 +639,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>604.4</t>
+          <t>280.3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>663.5</t>
+          <t>358.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>14.80</t>
+          <t>26.67</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -664,23 +664,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 📶</t>
+          <t xml:space="preserve"> By EbraSha 🔐</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>hysteria2</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>email protected:443</t>
+          <t>email protected:1001</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>636.2</t>
+          <t>365.4</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>634.1</t>
+          <t>284.2</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>638.3</t>
+          <t>446.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>15.65</t>
+          <t>20.83</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧠</t>
+          <t xml:space="preserve"> By EbraSha 🌀</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -731,17 +731,17 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>91.208.75.251:3478</t>
+          <t>series-a1.samanehha.co:443</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>647.6</t>
+          <t>365.5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>319.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -751,17 +751,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>577.7</t>
+          <t>219.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>717.6</t>
+          <t>511.1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>13.39</t>
+          <t>17.50</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🖥️</t>
+          <t xml:space="preserve"> By EbraSha 🩸</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -787,17 +787,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>140.174.184.5:8388</t>
+          <t>161.129.71.148:17913</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>662.9</t>
+          <t>390.4</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>14.8</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -807,17 +807,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>636.3</t>
+          <t>272.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>689.5</t>
+          <t>508.9</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>14.28</t>
+          <t>17.92</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -832,32 +832,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>By EbraSha 🕶️</t>
+          <t xml:space="preserve"> By EbraSha 📀</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>vmess</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>DE (Germany)</t>
-        </is>
-      </c>
+          <t>hysteria2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>89.167.82.102:4443</t>
+          <t>2001:19f0:7001:150:5400:6ff:fe44:1cfd:443</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>668.2</t>
+          <t>805.7</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>28.5</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -867,17 +863,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>389.8</t>
+          <t>404.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>946.6</t>
+          <t>1207.3</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.42</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -892,32 +888,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>By EbraSha 🚧</t>
+          <t xml:space="preserve"> By EbraSha 🔋</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>vmess</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DE (Germany)</t>
+          <t>??</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>89.167.82.102:4443</t>
+          <t>82.21.92.47:9443</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>670.2</t>
+          <t>821.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>30.7</t>
+          <t>743.4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -927,17 +923,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>412.5</t>
+          <t>796.5</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>927.9</t>
+          <t>845.6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>9.67</t>
+          <t>11.69</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -952,28 +948,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🔮</t>
+          <t xml:space="preserve"> By EbraSha 🔋</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>68.168.209.194:17276</t>
+          <t>162.249.126.198:443</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>673.2</t>
+          <t>1096.3</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>118.3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -983,17 +979,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>617.7</t>
+          <t>838.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>728.6</t>
+          <t>1353.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>13.30</t>
+          <t>6.85</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1024,12 +1020,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>681.0</t>
+          <t>1134.7</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>39.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1039,17 +1035,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>575.8</t>
+          <t>519.3</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>786.3</t>
+          <t>1750.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>12.05</t>
+          <t>4.99</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1064,28 +1060,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🦈</t>
+          <t xml:space="preserve"> By EbraSha ♣️</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>hysteria2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>109.73.65.116:493</t>
+          <t>2605:e440:10::1:68:443</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>728.6</t>
+          <t>1169.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1095,17 +1091,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>628.8</t>
+          <t>910.2</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>828.5</t>
+          <t>1427.8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>11.50</t>
+          <t>6.51</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1120,28 +1116,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🩸</t>
+          <t xml:space="preserve"> By EbraSha 🧊</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>161.129.71.148:17913</t>
+          <t>159.195.46.178:443</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>751.3</t>
+          <t>1260.8</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>130.9</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1151,17 +1147,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>707.5</t>
+          <t>1084.6</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>795.1</t>
+          <t>1437.0</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>12.30</t>
+          <t>6.62</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1176,28 +1172,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🥷</t>
+          <t xml:space="preserve"> By EbraSha 🌐</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>168.138.175.92:9888</t>
+          <t>95.85.233.181:443</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>760.8</t>
+          <t>1389.8</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>138.1</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1207,17 +1203,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>712.7</t>
+          <t>592.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>809.0</t>
+          <t>2186.9</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>12.06</t>
+          <t>3.97</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1232,28 +1228,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🔐</t>
+          <t xml:space="preserve"> By EbraSha ✨</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>email protected:1001</t>
+          <t>178.236.17.86:443</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>808.0</t>
+          <t>1636.5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>163.7</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1263,17 +1259,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>555.7</t>
+          <t>1434.6</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1060.2</t>
+          <t>1838.5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>8.59</t>
+          <t>5.20</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1288,28 +1284,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🕶️</t>
+          <t xml:space="preserve"> By EbraSha 🔌</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vless</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>email protected:8388</t>
+          <t>45.89.106.99:40443</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>808.1</t>
+          <t>1864.9</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>423.5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1319,17 +1315,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>705.1</t>
+          <t>1398.6</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>911.2</t>
+          <t>2331.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>10.48</t>
+          <t>3.96</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1344,28 +1340,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🚀</t>
+          <t xml:space="preserve"> By EbraSha ♠️</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>185.68.185.212:50029</t>
+          <t>email protected:17276</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>810.3</t>
+          <t>2166.5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1375,17 +1371,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>784.8</t>
+          <t>1213.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>835.8</t>
+          <t>3120.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>11.82</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1400,28 +1396,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🐺</t>
+          <t>US 🇺🇸 | @Raydikalx | 383</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>vmess</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>email protected:30129</t>
+          <t>57.151.100.27:10086</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>823.2</t>
+          <t>2381.2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>318.0</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1431,17 +1427,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>743.9</t>
+          <t>2080.5</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>902.4</t>
+          <t>2681.8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>10.69</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1456,7 +1452,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🧩</t>
+          <t xml:space="preserve"> By EbraSha 🤖</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1467,37 +1463,37 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>78.129.155.63:3030</t>
+          <t>ru.moktana.app:51523</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>857.2</t>
+          <t>221.4</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>137.8</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>576.4</t>
+          <t>221.4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1138.0</t>
+          <t>221.4</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>7.97</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1512,48 +1508,48 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> By EbraSha 🦅</t>
+          <t xml:space="preserve"> By EbraSha 🐉</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>77.73.131.154:443</t>
+          <t>admin.c1.webramz.co:443</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>907.8</t>
+          <t>240.6</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>345.5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>680.4</t>
+          <t>240.6</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1135.3</t>
+          <t>240.6</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>8.13</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1568,48 +1564,48 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>🎭</t>
+          <t xml:space="preserve"> By EbraSha 🦇</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>vless</t>
+          <t>ss</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>159.195.44.159:443</t>
+          <t>45.129.96.62:41348</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>920.1</t>
+          <t>269.7</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>153.1</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>670.4</t>
+          <t>269.7</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1169.8</t>
+          <t>269.7</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>7.85</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">

</xml_diff>